<commit_message>
20260528 solved problem with stod (lc_numeric)
</commit_message>
<xml_diff>
--- a/chemistry_book/content/project_THe/Group_Files/KR/tmp/df_work_PP-11N.xlsx
+++ b/chemistry_book/content/project_THe/Group_Files/KR/tmp/df_work_PP-11N.xlsx
@@ -460,19 +460,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>BB11N</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BoZ.CWZI-inf</t>
+          <t>PP-11N</t>
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>45022</v>
+        <v>46002</v>
       </c>
       <c r="D2" t="n">
-        <v>130</v>
+        <v>0.87</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -480,30 +480,30 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.003243512974051896</v>
+        <v>1.583545686203131e-05</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Ca+2.tot</t>
+          <t>Mn+2.tot</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>BB11N</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BoZ.CWZI-inf</t>
+          <t>PP-11N</t>
         </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>45022</v>
+        <v>46002</v>
       </c>
       <c r="D3" t="n">
-        <v>760</v>
+        <v>1</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -511,30 +511,30 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.03305785123966942</v>
+        <v>1.790510295434199e-05</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Na+.tot</t>
+          <t>Fe+2.tot</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>BB11N</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BoZ.CWZI-inf</t>
+          <t>PP-11N</t>
         </is>
       </c>
       <c r="C4" s="1" t="n">
-        <v>45022</v>
+        <v>46002</v>
       </c>
       <c r="D4" t="n">
-        <v>39.30871053141345</v>
+        <v>440</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -542,30 +542,30 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.0004139066076804617</v>
+        <v>0.01913875598086125</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>PO4-3.tot</t>
+          <t>Na+.tot</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>BB11N</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BoZ.CWZI-inf</t>
+          <t>PP-11N</t>
         </is>
       </c>
       <c r="C5" s="1" t="n">
-        <v>45022</v>
+        <v>46002</v>
       </c>
       <c r="D5" t="n">
-        <v>0.36</v>
+        <v>329.8627573300062</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -573,61 +573,61 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>6.55260283946123e-06</v>
+        <v>0.003433924186237833</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Mn+2.tot</t>
+          <t>SO4-2.tot</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>BB11N</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BoZ.CWZI-inf</t>
+          <t>PP-11N</t>
         </is>
       </c>
       <c r="C6" s="1" t="n">
-        <v>45022</v>
+        <v>46002</v>
       </c>
       <c r="D6" t="n">
-        <v>0.068</v>
+        <v>7.13</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>mg/l</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.120361708762083e-06</v>
+        <v>7.13</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>S-2.tot</t>
+          <t>pH</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>BB11N</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>BoZ.CWZI-inf</t>
+          <t>PP-11N</t>
         </is>
       </c>
       <c r="C7" s="1" t="n">
-        <v>45022</v>
+        <v>46002</v>
       </c>
       <c r="D7" t="n">
-        <v>6600</v>
+        <v>150.3734782608696</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -635,30 +635,30 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.1081612586037365</v>
+        <v>0.008335558661910733</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>HCO3-.tot</t>
+          <t>NH4+.tot</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>BB11N</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>BoZ.CWZI-inf</t>
+          <t>PP-11N</t>
         </is>
       </c>
       <c r="C8" s="1" t="n">
-        <v>45022</v>
+        <v>46002</v>
       </c>
       <c r="D8" t="n">
-        <v>500</v>
+        <v>0.1</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -666,30 +666,30 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.01278772378516624</v>
+        <v>3.118178983473652e-06</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>K+.tot</t>
+          <t>S-2.tot</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>BB11N</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>BoZ.CWZI-inf</t>
+          <t>PP-11N</t>
         </is>
       </c>
       <c r="C9" s="1" t="n">
-        <v>45022</v>
+        <v>46002</v>
       </c>
       <c r="D9" t="n">
-        <v>6.7</v>
+        <v>21</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -697,30 +697,30 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.0001199641897940913</v>
+        <v>0.0007475970096119616</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Fe+2.tot</t>
+          <t>Si.tot</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>BB11N</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>BoZ.CWZI-inf</t>
+          <t>PP-11N</t>
         </is>
       </c>
       <c r="C10" s="1" t="n">
-        <v>45022</v>
+        <v>46002</v>
       </c>
       <c r="D10" t="n">
-        <v>92</v>
+        <v>460</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -728,30 +728,30 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.0009577347491151364</v>
+        <v>0.01147704590818363</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>SO4-2.tot</t>
+          <t>Ca+2.tot</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>BB11N</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>BoZ.CWZI-inf</t>
+          <t>PP-11N</t>
         </is>
       </c>
       <c r="C11" s="1" t="n">
-        <v>45022</v>
+        <v>46002</v>
       </c>
       <c r="D11" t="n">
-        <v>23.6</v>
+        <v>507</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -759,61 +759,61 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.0008401566393734426</v>
+        <v>0.01430183356840621</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Si.tot</t>
+          <t>Cl-.tot</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>BB11N</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>BoZ.CWZI-inf</t>
+          <t>PP-11N</t>
         </is>
       </c>
       <c r="C12" s="1" t="n">
-        <v>45022</v>
+        <v>46002</v>
       </c>
       <c r="D12" t="n">
-        <v>7.6</v>
+        <v>11.25</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>mg/l</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>7.6</v>
+        <v>0.0001184584605664947</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>pH</t>
+          <t>PO4-3.tot</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>BB11N</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BoZ.CWZI-inf</t>
+          <t>PP-11N</t>
         </is>
       </c>
       <c r="C13" s="1" t="n">
-        <v>45022</v>
+        <v>46002</v>
       </c>
       <c r="D13" t="n">
-        <v>55</v>
+        <v>3800</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -821,30 +821,30 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.002262443438914027</v>
+        <v>0.06227466404457555</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Mg+2.tot</t>
+          <t>HCO3-.tot</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>BB11N</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BoZ.CWZI-inf</t>
+          <t>PP-11N</t>
         </is>
       </c>
       <c r="C14" s="1" t="n">
-        <v>45022</v>
+        <v>46002</v>
       </c>
       <c r="D14" t="n">
-        <v>1192.413793103448</v>
+        <v>180</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -852,55 +852,73 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.0660983255600581</v>
+        <v>0.007404360345536817</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>NH4+.tot</t>
+          <t>Mg+2.tot</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>BB11N</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>BoZ.CWZI-inf</t>
+          <t>PP-11N</t>
         </is>
       </c>
       <c r="C15" s="1" t="n">
-        <v>45022</v>
+        <v>46002</v>
       </c>
       <c r="D15" t="n">
-        <v>850</v>
+        <v>14.7</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>mg/l</t>
+          <t>°C</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.02397743300423131</v>
+        <v>287.85</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Cl-.tot</t>
+          <t>T</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>BB11N</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>PP-11N</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="n">
+        <v>46002</v>
+      </c>
+      <c r="D16" t="n">
+        <v>210</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>mg/l</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>0.005370843989769821</v>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>K+.tot</t>
         </is>
       </c>
     </row>

</xml_diff>